<commit_message>
Correct DSO cash release calculation
</commit_message>
<xml_diff>
--- a/02-working-capital-aging-analyzer/excel/working_capital_analyzer.xlsx
+++ b/02-working-capital-aging-analyzer/excel/working_capital_analyzer.xlsx
@@ -1189,7 +1189,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>306666.6666666667</t>
+          <t>237500.0</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>110000.0</t>
+          <t>85190.22</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>40833.33</t>
+          <t>31623.64</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>63333.33</t>
+          <t>49048.91</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>49166.67</t>
+          <t>38077.45</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>43333.33</t>
+          <t>33559.78</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1925,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>110000.0</t>
+          <t>85190.22</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>40833.33</t>
+          <t>31623.64</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>63333.33</t>
+          <t>49048.91</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>49166.67</t>
+          <t>38077.45</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>43333.33</t>
+          <t>33559.78</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">

</xml_diff>